<commit_message>
feat(templates_base): house_style 베이스 템플릿 10종 + unit_economics 수식 방어
- tools/make_base_templates.py: 골든샘플에서 입력셀(파랑)만 비운 베이스 .xlsx 생성
  (채우기모드 캔버스 + Excel 에서 스파크라인/조건부서식 덧입힐 출발점). 자작본(라이선스 무관).
- templates_base/<type>_base.xlsx 10종 — 전부 Excel COM 재계산 0에러 검증.
- fix(unit_economics): 고객수명 ''(churn=0/미입력) 시 LTV 텍스트곱셈 #VALUE! 방어
  (IF 가드 추가). 회귀: selftest ALL PASS, unittest 9/9, Excel 재검증 OK.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/unit_economics_golden.xlsx
+++ b/samples/unit_economics_golden.xlsx
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>B5*B6*B11</f>
+        <f>IF(B11="","",B5*B6*B11)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>IF(B8=0,"",B12/B8)</f>
+        <f>IF(OR(B8=0,B12=""),"",B12/B8)</f>
         <v/>
       </c>
     </row>

</xml_diff>